<commit_message>
CORE-000535 edit: test data updated
</commit_message>
<xml_diff>
--- a/rules/CORE-000535/negative/01/data/unit-test-coreid-CG0620-negative 1.xlsx
+++ b/rules/CORE-000535/negative/01/data/unit-test-coreid-CG0620-negative 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\CORE-000535\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40562809-E9A4-4A7F-A09D-84C01D1CD8FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C7348A-E61F-42DA-9E06-4F94F01181D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="555" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{68203D44-07AE-4443-B366-E6DFDE0510A4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21240" windowHeight="15270" activeTab="2" xr2:uid="{68203D44-07AE-4443-B366-E6DFDE0510A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="4" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="79">
   <si>
     <t>Product</t>
   </si>
@@ -344,7 +344,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -364,24 +364,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEDEDED"/>
-        <bgColor rgb="FFEDEDED"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFEDEDED"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="4">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -434,20 +422,126 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="6"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="6"/>
+      </left>
+      <right style="thin">
+        <color theme="6"/>
+      </right>
+      <top style="thin">
+        <color theme="6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="6"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color theme="6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="6"/>
+      </left>
+      <right style="thin">
+        <color theme="6"/>
+      </right>
+      <top style="medium">
+        <color theme="6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="6"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="6"/>
+      </top>
+      <bottom style="thin">
+        <color theme="6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="6"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="6"/>
+      </left>
+      <right style="thin">
+        <color theme="6"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -455,38 +549,92 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -494,56 +642,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Note" xfId="1" builtinId="10"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -554,45 +653,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{75188EF8-0D12-4113-9C59-BB606E98A87F}" name="Table38293755586162" displayName="Table38293755586162" ref="A1:K6" totalsRowShown="0">
-  <autoFilter ref="A1:K6" xr:uid="{75188EF8-0D12-4113-9C59-BB606E98A87F}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{CAFA8D04-1FD1-4FC4-8FD8-EBED212015FE}" name="STUDYID"/>
-    <tableColumn id="2" xr3:uid="{437B7FC3-9D6B-44F0-A379-B7990E0B35E2}" name="DOMAIN"/>
-    <tableColumn id="3" xr3:uid="{6D28D649-E2DF-4516-B97F-C947C3E99EAA}" name="USUBJID"/>
-    <tableColumn id="4" xr3:uid="{32E70E5A-B346-4260-A652-7B46DACD0114}" name="SESEQ"/>
-    <tableColumn id="5" xr3:uid="{4F00841E-F6C2-4A85-AA8E-79AF2758E63F}" name="ETCD"/>
-    <tableColumn id="6" xr3:uid="{DD7937A0-CA66-4C1A-9C0B-95FD02778B0F}" name="ELEMENT"/>
-    <tableColumn id="7" xr3:uid="{084DD905-A4D3-497B-922E-B0D87DD821ED}" name="EPOCH"/>
-    <tableColumn id="8" xr3:uid="{00C50A7B-7CDF-4EEA-B76F-84EF5CCFF395}" name="SESTDTC"/>
-    <tableColumn id="9" xr3:uid="{DBE620CD-DEBB-49BC-A883-550BA4EEB05D}" name="SEENDTC"/>
-    <tableColumn id="10" xr3:uid="{E366C12D-5625-4DAD-BD2A-13FE075ED474}" name="SESTDY"/>
-    <tableColumn id="11" xr3:uid="{34AC7978-EB9E-4A6C-999C-813162618C3F}" name="SEENDY"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D4C2B4A4-1709-4E54-A7E4-CBEB4CB799C7}" name="Table38293743505152" displayName="Table38293743505152" ref="A1:J12" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J12" xr:uid="{00000000-0009-0000-0100-000033000000}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{545C8250-1183-44BC-9DC6-53F5FD6FABCF}" name="STUDYID" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{F0651F9A-81E2-47C0-BD58-92DF7041654D}" name="DOMAIN" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{16A18C95-C0C0-4533-B772-79BE192BFFA3}" name="USUBJID" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{55ED61B5-8440-4D5D-A6B0-B5CDA710AF93}" name="SMSEQ" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{F0378F8A-7685-4E19-AECE-73F26CE5175A}" name="MIDS" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{03A0A831-88BF-4C93-8C4D-1AC9381C03F7}" name="MIDSTYPE" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{DDE327B6-A8EE-43A0-BC17-F1656439CF0A}" name="SMSTDTC" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{8951F9A4-F335-49D1-8287-07ABDC438BDB}" name="SMENDTC" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{E63804E9-6478-4EFE-9B2D-01F9826FFB14}" name="SMSTDY" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{6EAB0783-0CFF-4264-BF6E-F88BECD8B95B}" name="SMENDY" dataDxfId="0"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -907,7 +967,7 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>3</v>
       </c>
     </row>
@@ -925,18 +985,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -955,29 +1015,29 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68BEEBCD-2776-477F-B12E-85A72C199137}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="6" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1001,7 +1061,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1017,7 +1077,7 @@
       <c r="E3" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="1" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1057,7 +1117,7 @@
       <c r="E5" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="1" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1065,279 +1125,239 @@
       <c r="A6">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C6" t="s">
         <v>78</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6" t="s">
         <v>43</v>
       </c>
-      <c r="F6">
-        <v>1</v>
+      <c r="F6" s="7">
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C7" t="s">
         <v>78</v>
       </c>
       <c r="D7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E7" t="s">
         <v>46</v>
       </c>
-      <c r="F7" s="18" t="s">
-        <v>61</v>
+      <c r="F7" s="1" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C8" t="s">
         <v>78</v>
       </c>
       <c r="D8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E8" t="s">
         <v>43</v>
       </c>
-      <c r="F8" s="5">
-        <v>2</v>
+      <c r="F8" s="7">
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>4</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C9" t="s">
         <v>78</v>
       </c>
       <c r="D9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E9" t="s">
         <v>46</v>
       </c>
-      <c r="F9" s="18" t="s">
-        <v>62</v>
+      <c r="F9" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>5</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C10" t="s">
         <v>78</v>
       </c>
       <c r="D10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E10" t="s">
         <v>43</v>
       </c>
-      <c r="F10" s="5">
-        <v>3</v>
+      <c r="F10">
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>5</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C11" t="s">
         <v>78</v>
       </c>
       <c r="D11">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E11" t="s">
         <v>46</v>
       </c>
-      <c r="F11" s="18" t="s">
-        <v>63</v>
+      <c r="F11" s="1" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>6</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C12" t="s">
         <v>78</v>
       </c>
       <c r="D12">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E12" t="s">
         <v>43</v>
       </c>
       <c r="F12">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>6</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C13" t="s">
         <v>78</v>
       </c>
       <c r="D13">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E13" t="s">
         <v>46</v>
       </c>
-      <c r="F13" s="18" t="s">
-        <v>66</v>
+      <c r="F13" s="1" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>7</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C14" t="s">
         <v>78</v>
       </c>
       <c r="D14">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E14" t="s">
         <v>43</v>
       </c>
       <c r="F14">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>7</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C15" t="s">
         <v>78</v>
       </c>
       <c r="D15">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E15" t="s">
         <v>46</v>
       </c>
-      <c r="F15" s="18" t="s">
-        <v>70</v>
+      <c r="F15" s="1" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>8</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C16" t="s">
         <v>78</v>
       </c>
       <c r="D16">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E16" t="s">
         <v>43</v>
       </c>
       <c r="F16">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>8</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C17" t="s">
         <v>78</v>
       </c>
       <c r="D17">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E17" t="s">
         <v>46</v>
       </c>
-      <c r="F17" s="18" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>9</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C18" t="s">
-        <v>78</v>
-      </c>
-      <c r="D18">
-        <v>12</v>
-      </c>
-      <c r="E18" t="s">
-        <v>43</v>
-      </c>
-      <c r="F18">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>9</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C19" t="s">
-        <v>78</v>
-      </c>
-      <c r="D19">
-        <v>12</v>
-      </c>
-      <c r="E19" t="s">
-        <v>46</v>
-      </c>
-      <c r="F19" s="18" t="s">
+      <c r="F17" s="1" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1349,7 +1369,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4BFCEED-7F72-45AA-AEFF-7CE85C6A47FC}">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
@@ -1364,234 +1384,218 @@
     <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="9" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="11" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="13" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
+      <c r="A4" s="12">
         <v>50</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="12">
         <v>50</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="12">
         <v>50</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="12">
         <v>8</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="12">
         <v>50</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="12">
         <v>50</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="12">
         <v>50</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="12">
         <v>50</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="12">
         <v>50</v>
       </c>
-      <c r="J4" s="8">
+      <c r="J4" s="12">
         <v>8</v>
       </c>
-      <c r="K4" s="8">
+      <c r="K4" s="13">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="14" t="s">
         <v>36</v>
       </c>
       <c r="D5" s="15">
         <v>2</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="H5" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="14">
         <v>-7</v>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="18">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="23">
         <v>1</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="H6" s="14" t="s">
+      <c r="H6" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="J6" s="10">
+      <c r="J6" s="20">
         <v>1</v>
       </c>
-      <c r="K6" s="10">
+      <c r="K6" s="22">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="11"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -1605,338 +1609,349 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="25" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="27" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="27" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+      <c r="A4" s="26">
         <v>50</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="26">
         <v>50</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="26">
         <v>50</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="26">
         <v>8</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="26">
         <v>50</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="26">
         <v>50</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="26">
         <v>50</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="26">
         <v>50</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="26">
         <v>8</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="27">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="35">
         <v>1</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="28" t="s">
         <v>61</v>
       </c>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="31"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="29">
         <v>2</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G6" s="16" t="s">
         <v>62</v>
       </c>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="33"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="29">
         <v>3</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="16" t="s">
         <v>63</v>
       </c>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="33"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="29">
         <v>5</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="16" t="s">
         <v>66</v>
       </c>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="33"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="32">
         <v>1</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="17" t="s">
         <v>71</v>
       </c>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="33"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="29">
         <v>3</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="G10" s="16" t="s">
         <v>70</v>
       </c>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="33"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="29">
         <v>4</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="16" t="s">
         <v>67</v>
       </c>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="33"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="30">
         <v>2</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="G12" s="14" t="s">
+      <c r="G12" s="19" t="s">
         <v>68</v>
       </c>
+      <c r="H12" s="21"/>
+      <c r="I12" s="21"/>
+      <c r="J12" s="34"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId2"/>
-  </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Comment xmlns="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010090ADB40D834AE945B19FCDA4041AC0CB" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d36826f407302d9fd93d8089214679b0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xmlns:ns3="63ea592b-d684-45c7-8cdc-fad8f8e6bb41" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="257daeb82d9c284d9d656fb5e9ad601e" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -2176,7 +2191,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2185,25 +2200,17 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A3465CB0-AE5A-4E05-8903-7C175B9B106D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="63ea592b-d684-45c7-8cdc-fad8f8e6bb41"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Comment xmlns="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F6B15BE-5C05-4CD5-9B66-DE4C08005052}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2223,10 +2230,28 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F29E9FB3-078C-46A0-ACEC-1E7A83B21788}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A3465CB0-AE5A-4E05-8903-7C175B9B106D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="63ea592b-d684-45c7-8cdc-fad8f8e6bb41"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>